<commit_message>
Change in sortBiMileagePage waits given for sleep
</commit_message>
<xml_diff>
--- a/ExcelData/report.xlsx
+++ b/ExcelData/report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="27">
   <si>
     <t>Sr. No.</t>
   </si>
@@ -85,6 +85,15 @@
   </si>
   <si>
     <t>NAME: Bajaj Pulsar NS400Z | RATING: 4.6/5 (106 Ratings) | SPECS: 373 cc|32 kmpl|42.41 bhp|174 kg | PRICE: ₹ 1,94,061</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj CT 110 | RATING: 4.4/5 (115 Ratings) | SPECS: 115.45 cc|70 kmpl|8.48 bhp|127 kg | PRICE: ₹ 68,050</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Platina 110 | RATING: 4.4/5 (170 Ratings) | SPECS: 115.45 cc|70 kmpl|8.48 bhp|119 kg | PRICE: ₹ 69,941</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Pulsar 150 | RATING: 4.5/5 (1428 Ratings) | SPECS: 149.5 cc|49 kmpl|13.8 bhp|148 kg | PRICE: ₹ 1,10,120</t>
   </si>
 </sst>
 </file>
@@ -369,7 +378,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +474,7 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -473,7 +482,7 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Adding test-ouput file and make changes in xpath for brandList in TC_01
</commit_message>
<xml_diff>
--- a/ExcelData/report.xlsx
+++ b/ExcelData/report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="30">
   <si>
     <t>Sr. No.</t>
   </si>
@@ -94,6 +94,15 @@
   </si>
   <si>
     <t>NAME: Bajaj Pulsar 150 | RATING: 4.5/5 (1428 Ratings) | SPECS: 149.5 cc|49 kmpl|13.8 bhp|148 kg | PRICE: ₹ 1,10,120</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Pulsar N160 | RATING: 4.6/5 (285 Ratings) | SPECS: 164.82 cc|51.6 kmpl|15.68 bhp|152 kg | PRICE: ₹ 1,14,840</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Avenger Cruise 220 | RATING: 4.4/5 (341 Ratings) | SPECS: 220 cc|39 kmpl|18.76 bhp|163 kg | PRICE: ₹ 1,26,620</t>
+  </si>
+  <si>
+    <t>NAME: Bajaj Pulsar N125 | RATING: 4.4/5 (38 Ratings) | SPECS: 124.58 cc|60 kmpl|11.83 bhp|125 kg | PRICE: ₹ 93,668</t>
   </si>
 </sst>
 </file>
@@ -338,7 +347,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +443,7 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>14</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -458,7 +467,7 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18">

</xml_diff>